<commit_message>
Save changed before syncing
</commit_message>
<xml_diff>
--- a/HV Module Test/hv_module_test_dry_run.xlsx
+++ b/HV Module Test/hv_module_test_dry_run.xlsx
@@ -17,7 +17,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="3">
+  <fonts count="4">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -30,6 +30,9 @@
     </font>
     <font>
       <color rgb="00009900"/>
+    </font>
+    <font>
+      <color rgb="00FF0000"/>
     </font>
   </fonts>
   <fills count="2">
@@ -52,10 +55,11 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -421,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AW2"/>
+  <dimension ref="A1:AW4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -911,6 +915,496 @@
         </is>
       </c>
       <c r="AW2" s="2" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>dry_run</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>09/10/2026</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>06:03:09 PM</t>
+        </is>
+      </c>
+      <c r="D3" t="n">
+        <v>2</v>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>E08F2</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>DRYRUN123</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>07.52</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>negative</t>
+        </is>
+      </c>
+      <c r="I3" s="3" t="inlineStr">
+        <is>
+          <t>FAIL</t>
+        </is>
+      </c>
+      <c r="J3" s="2" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="K3" s="2" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="L3" s="2" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="M3" s="2" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="N3" s="2" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="O3" s="2" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="P3" s="2" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="Q3" s="2" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="R3" s="2" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="S3" s="2" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="T3" s="2" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="U3" s="2" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="V3" s="2" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="W3" s="2" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="X3" s="2" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="Y3" s="2" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="Z3" s="2" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="AA3" s="3" t="inlineStr">
+        <is>
+          <t>FAIL</t>
+        </is>
+      </c>
+      <c r="AB3" s="2" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="AC3" s="2" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="AD3" s="2" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="AE3" s="2" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="AF3" s="2" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="AG3" s="2" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="AH3" s="3" t="inlineStr">
+        <is>
+          <t>FAIL</t>
+        </is>
+      </c>
+      <c r="AI3" s="2" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="AJ3" s="2" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="AK3" s="2" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="AL3" s="2" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="AM3" s="2" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="AN3" s="2" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="AO3" s="2" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="AP3" s="2" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="AQ3" s="2" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="AR3" s="2" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="AS3" s="2" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="AT3" s="2" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="AU3" s="2" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="AV3" s="2" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="AW3" s="2" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>dry_run</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>09/10/2026</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>06:05:02 PM</t>
+        </is>
+      </c>
+      <c r="D4" t="n">
+        <v>2</v>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>E08F2</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>DRYRUN123</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>07.52</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>negative</t>
+        </is>
+      </c>
+      <c r="I4" s="2" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="J4" s="2" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="K4" s="2" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="L4" s="2" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="M4" s="2" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="N4" s="2" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="O4" s="2" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="P4" s="2" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="Q4" s="2" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="R4" s="2" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="S4" s="2" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="T4" s="2" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="U4" s="2" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="V4" s="2" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="W4" s="2" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="X4" s="2" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="Y4" s="2" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="Z4" s="2" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="AA4" s="2" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="AB4" s="2" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="AC4" s="2" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="AD4" s="2" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="AE4" s="2" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="AF4" s="2" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="AG4" s="2" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="AH4" s="2" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="AI4" s="2" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="AJ4" s="2" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="AK4" s="2" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="AL4" s="2" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="AM4" s="2" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="AN4" s="2" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="AO4" s="2" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="AP4" s="2" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="AQ4" s="2" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="AR4" s="2" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="AS4" s="2" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="AT4" s="2" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="AU4" s="2" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="AV4" s="2" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="AW4" s="2" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>

</xml_diff>

<commit_message>
Moved WIB WIEC testing files into WIEC components folder, working on integration with the WIEC components API.
Changing logic of the WIB WIEC testing to be that wiec_wib_qc is the top file, and the others are helpers that handle one WIB at a time instead of all at once. This allows for desired testing process of moving between WIBs in the crate.

Not in a working state.
</commit_message>
<xml_diff>
--- a/HV Module Test/hv_module_test_dry_run.xlsx
+++ b/HV Module Test/hv_module_test_dry_run.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AW4"/>
+  <dimension ref="A1:AZ6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -674,6 +674,21 @@
           <t>HV Limit Readback</t>
         </is>
       </c>
+      <c r="AX1" s="1" t="inlineStr">
+        <is>
+          <t>HV I-V Measurement</t>
+        </is>
+      </c>
+      <c r="AY1" s="1" t="inlineStr">
+        <is>
+          <t>HV I-V Linearity</t>
+        </is>
+      </c>
+      <c r="AZ1" s="1" t="inlineStr">
+        <is>
+          <t>HV I-V Channel Uniformity</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -1405,6 +1420,526 @@
         </is>
       </c>
       <c r="AW4" s="2" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>dry_run</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>09/23/2026</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>07:00:46 PM</t>
+        </is>
+      </c>
+      <c r="D5" t="n">
+        <v>2</v>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>E08F2</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>DRYRUN123</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>07.52</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>negative</t>
+        </is>
+      </c>
+      <c r="I5" s="2" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="J5" s="2" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="K5" s="2" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="L5" s="2" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="M5" s="2" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="N5" s="2" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="O5" s="2" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="P5" s="2" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="Q5" s="2" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="R5" s="2" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="S5" s="2" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="T5" s="2" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="U5" s="2" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="V5" s="2" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="W5" s="2" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="X5" s="2" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="Y5" s="2" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="Z5" s="2" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="AA5" s="2" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="AB5" s="2" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="AC5" s="2" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="AD5" s="2" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="AE5" s="2" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="AF5" s="2" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="AG5" s="2" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="AH5" s="2" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="AI5" s="2" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="AJ5" s="2" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="AK5" s="2" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="AL5" s="2" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="AM5" s="2" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="AN5" s="2" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="AO5" s="2" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="AP5" s="2" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="AQ5" s="2" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="AR5" s="2" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="AS5" s="2" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="AT5" s="2" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="AU5" s="2" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="AV5" s="2" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="AW5" s="2" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="AX5" s="2" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="AY5" s="2" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="AZ5" s="2" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>dry_run</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>09/23/2026</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>07:03:09 PM</t>
+        </is>
+      </c>
+      <c r="D6" t="n">
+        <v>2</v>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>E08F2</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>DRYRUN123</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>07.52</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>negative</t>
+        </is>
+      </c>
+      <c r="I6" s="2" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="J6" s="2" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="K6" s="2" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="L6" s="2" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="M6" s="2" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="N6" s="2" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="O6" s="2" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="P6" s="2" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="Q6" s="2" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="R6" s="2" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="S6" s="2" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="T6" s="2" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="U6" s="2" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="V6" s="2" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="W6" s="2" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="X6" s="2" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="Y6" s="2" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="Z6" s="2" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="AA6" s="2" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="AB6" s="2" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="AC6" s="2" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="AD6" s="2" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="AE6" s="2" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="AF6" s="2" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="AG6" s="2" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="AH6" s="2" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="AI6" s="2" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="AJ6" s="2" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="AK6" s="2" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="AL6" s="2" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="AM6" s="2" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="AN6" s="2" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="AO6" s="2" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="AP6" s="2" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="AQ6" s="2" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="AR6" s="2" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="AS6" s="2" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="AT6" s="2" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="AU6" s="2" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="AV6" s="2" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="AW6" s="2" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="AX6" s="2" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="AY6" s="2" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="AZ6" s="2" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>

</xml_diff>